<commit_message>
Update: Added Loan - Web scenarios.
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/EnterpriseTestData.xlsx
+++ b/src/test/resources/testdata/EnterpriseTestData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/7717805a7dbae679/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="5" documentId="11_84B3479C16D7A9B5D87DA434AA0045C33F72AACB" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{64C5B924-BC47-4332-A97B-D28782A7414C}"/>
+  <xr:revisionPtr revIDLastSave="29" documentId="11_84B3479C16D7A9B5D87DA434AA0045C33F72AACB" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5D7D6596-007F-4F34-AACA-1746CB32E5DE}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="5" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="5" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="LoginData" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="88">
   <si>
     <t>TestCaseID</t>
   </si>
@@ -277,13 +277,22 @@
     <t>Loan_001</t>
   </si>
   <si>
-    <t>5000</t>
-  </si>
-  <si>
-    <t>500</t>
-  </si>
-  <si>
-    <t>Loan request within typical approval range</t>
+    <t>Approved</t>
+  </si>
+  <si>
+    <t>Small loan amount reliably approved</t>
+  </si>
+  <si>
+    <t>ExpectedStatus</t>
+  </si>
+  <si>
+    <t>Loan_002</t>
+  </si>
+  <si>
+    <t>Denied</t>
+  </si>
+  <si>
+    <t>Large loan amount reliably denied due to insufficient funds</t>
   </si>
 </sst>
 </file>
@@ -767,15 +776,18 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="2" width="12" customWidth="1"/>
-    <col min="3" max="4" width="14" customWidth="1"/>
-    <col min="5" max="5" width="44" customWidth="1"/>
+    <col min="1" max="1" width="12.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.21875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.77734375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="52.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -788,25 +800,51 @@
       <c r="D1" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="F1" s="3" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="4">
+        <v>100</v>
+      </c>
+      <c r="C2" s="4">
+        <v>10</v>
+      </c>
+      <c r="D2" s="4">
+        <v>12567</v>
+      </c>
+      <c r="E2" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="F2" t="s">
         <v>83</v>
       </c>
-      <c r="D2" s="4">
-        <v>22224</v>
-      </c>
-      <c r="E2" t="s">
-        <v>84</v>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="B3" s="4">
+        <v>10000</v>
+      </c>
+      <c r="C3" s="4">
+        <v>10</v>
+      </c>
+      <c r="D3" s="4">
+        <v>12567</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="F3" t="s">
+        <v>87</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added: Register New User - Web Scenarios.
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/EnterpriseTestData.xlsx
+++ b/src/test/resources/testdata/EnterpriseTestData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/7717805a7dbae679/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="30" documentId="11_84B3479C16D7A9B5D87DA434AA0045C33F72AACB" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{998CFB94-CAD1-4E6E-99CB-ED0B1229BA87}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="11_A180A8D17879FCD29DF161CB5464D75B08B36FDF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A10309DB-2934-4B9A-9157-FF2D155A5BAA}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="7" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="7" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="LoginData" sheetId="1" r:id="rId1"/>
@@ -23,26 +23,57 @@
     <sheet name="BillPayData" sheetId="8" r:id="rId8"/>
     <sheet name="UpdateContactData" sheetId="9" r:id="rId9"/>
     <sheet name="RequestLoanData" sheetId="10" r:id="rId10"/>
+    <sheet name="RegisterData" sheetId="11" r:id="rId11"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="101">
   <si>
     <t>TestCaseID</t>
   </si>
   <si>
+    <t>LoanAmount</t>
+  </si>
+  <si>
+    <t>DownPayment</t>
+  </si>
+  <si>
+    <t>FromAccount</t>
+  </si>
+  <si>
+    <t>ExpectedStatus</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>Loan_001</t>
+  </si>
+  <si>
+    <t>Approved</t>
+  </si>
+  <si>
+    <t>Small loan amount reliably approved</t>
+  </si>
+  <si>
+    <t>Loan_002</t>
+  </si>
+  <si>
+    <t>Denied</t>
+  </si>
+  <si>
+    <t>Large loan amount reliably denied due to insufficient funds</t>
+  </si>
+  <si>
     <t>Username</t>
   </si>
   <si>
     <t>Password</t>
   </si>
   <si>
-    <t>Description</t>
-  </si>
-  <si>
     <t>Login_001</t>
   </si>
   <si>
@@ -79,9 +110,6 @@
     <t>Valid account iteration 3</t>
   </si>
   <si>
-    <t>FromAccount</t>
-  </si>
-  <si>
     <t>ToAccount</t>
   </si>
   <si>
@@ -268,31 +296,43 @@
     <t>Update all contact fields with valid values</t>
   </si>
   <si>
-    <t>LoanAmount</t>
-  </si>
-  <si>
-    <t>DownPayment</t>
-  </si>
-  <si>
-    <t>Loan_001</t>
-  </si>
-  <si>
-    <t>Approved</t>
-  </si>
-  <si>
-    <t>Small loan amount reliably approved</t>
-  </si>
-  <si>
-    <t>ExpectedStatus</t>
-  </si>
-  <si>
-    <t>Loan_002</t>
-  </si>
-  <si>
-    <t>Denied</t>
-  </si>
-  <si>
-    <t>Large loan amount reliably denied due to insufficient funds</t>
+    <t>SSN</t>
+  </si>
+  <si>
+    <t>Register_001</t>
+  </si>
+  <si>
+    <t>Alex</t>
+  </si>
+  <si>
+    <t>Morgan</t>
+  </si>
+  <si>
+    <t>789 Enroll Ave</t>
+  </si>
+  <si>
+    <t>Austin</t>
+  </si>
+  <si>
+    <t>Texas</t>
+  </si>
+  <si>
+    <t>73301</t>
+  </si>
+  <si>
+    <t>5125550101</t>
+  </si>
+  <si>
+    <t>987654321</t>
+  </si>
+  <si>
+    <t>SecurePass!23</t>
+  </si>
+  <si>
+    <t>New user registration with unique runtime-suffixed username</t>
+  </si>
+  <si>
+    <t>qa_morganalex_99_</t>
   </si>
 </sst>
 </file>
@@ -381,10 +421,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -717,55 +753,55 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>2</v>
+        <v>13</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>7</v>
+        <v>17</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>11</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>13</v>
+        <v>23</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>15</v>
+        <v>25</v>
       </c>
     </row>
   </sheetData>
@@ -792,24 +828,24 @@
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>79</v>
+        <v>1</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>16</v>
+        <v>3</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>84</v>
+        <v>4</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
-        <v>81</v>
+        <v>6</v>
       </c>
       <c r="B2" s="4">
         <v>100</v>
@@ -821,15 +857,15 @@
         <v>12567</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>82</v>
+        <v>7</v>
       </c>
       <c r="F2" t="s">
-        <v>83</v>
+        <v>8</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
-        <v>85</v>
+        <v>9</v>
       </c>
       <c r="B3" s="4">
         <v>100000000</v>
@@ -841,10 +877,108 @@
         <v>12567</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>86</v>
+        <v>10</v>
       </c>
       <c r="F3" t="s">
-        <v>87</v>
+        <v>11</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
+  <dimension ref="A1:L2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="3" width="12" customWidth="1"/>
+    <col min="4" max="4" width="18" customWidth="1"/>
+    <col min="5" max="5" width="12" customWidth="1"/>
+    <col min="6" max="7" width="10" customWidth="1"/>
+    <col min="8" max="8" width="14" customWidth="1"/>
+    <col min="9" max="9" width="12" customWidth="1"/>
+    <col min="10" max="10" width="20.77734375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="16" customWidth="1"/>
+    <col min="12" max="12" width="50" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="K1" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="L1" s="3" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A2" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="H2" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="I2" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="J2" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="K2" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="L2" s="4" t="s">
+        <v>99</v>
       </c>
     </row>
   </sheetData>
@@ -871,33 +1005,33 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>2</v>
+        <v>13</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>16</v>
+        <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>17</v>
+        <v>26</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="D2" s="2">
         <v>22224</v>
@@ -909,18 +1043,18 @@
         <v>10</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>20</v>
+        <v>29</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="D3" s="2">
         <v>56634</v>
@@ -932,7 +1066,7 @@
         <v>25.5</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>22</v>
+        <v>31</v>
       </c>
     </row>
   </sheetData>
@@ -957,50 +1091,50 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>2</v>
+        <v>13</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>16</v>
+        <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
-        <v>23</v>
+        <v>32</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="D2" s="2">
         <v>22224</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>24</v>
+        <v>33</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
-        <v>25</v>
+        <v>34</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="D3" s="2">
         <v>56634</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>26</v>
+        <v>35</v>
       </c>
     </row>
   </sheetData>
@@ -1023,55 +1157,55 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>2</v>
+        <v>13</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>7</v>
+        <v>17</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>11</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>13</v>
+        <v>23</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>15</v>
+        <v>25</v>
       </c>
     </row>
   </sheetData>
@@ -1096,41 +1230,41 @@
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>27</v>
+        <v>36</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>28</v>
+        <v>37</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
-        <v>29</v>
+        <v>38</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="C2" s="4">
         <v>2</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>31</v>
+        <v>40</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
-        <v>32</v>
+        <v>41</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>33</v>
+        <v>42</v>
       </c>
       <c r="C3" s="4">
         <v>1</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>34</v>
+        <v>43</v>
       </c>
     </row>
   </sheetData>
@@ -1161,81 +1295,81 @@
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>27</v>
+        <v>36</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>28</v>
+        <v>37</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>35</v>
+        <v>44</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>36</v>
+        <v>45</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>37</v>
+        <v>46</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>38</v>
+        <v>47</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>40</v>
+        <v>49</v>
       </c>
       <c r="J1" s="3" t="s">
-        <v>41</v>
+        <v>50</v>
       </c>
       <c r="K1" s="3" t="s">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="L1" s="3" t="s">
-        <v>43</v>
+        <v>52</v>
       </c>
       <c r="M1" s="3" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="C2" s="4">
         <v>1</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>45</v>
+        <v>54</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>46</v>
+        <v>55</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>47</v>
+        <v>56</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>48</v>
+        <v>57</v>
       </c>
       <c r="H2" s="4" t="s">
-        <v>49</v>
+        <v>58</v>
       </c>
       <c r="I2" s="4" t="s">
-        <v>50</v>
+        <v>59</v>
       </c>
       <c r="J2" s="4" t="s">
-        <v>51</v>
+        <v>60</v>
       </c>
       <c r="K2" s="4" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="L2" s="4" t="s">
-        <v>53</v>
+        <v>62</v>
       </c>
       <c r="M2" s="4" t="s">
-        <v>54</v>
+        <v>63</v>
       </c>
     </row>
   </sheetData>
@@ -1267,93 +1401,93 @@
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>27</v>
+        <v>36</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>28</v>
+        <v>37</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>2</v>
+        <v>13</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>35</v>
+        <v>44</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>36</v>
+        <v>45</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>37</v>
+        <v>46</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>38</v>
+        <v>47</v>
       </c>
       <c r="J1" s="3" t="s">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="K1" s="3" t="s">
-        <v>40</v>
+        <v>49</v>
       </c>
       <c r="L1" s="3" t="s">
-        <v>41</v>
+        <v>50</v>
       </c>
       <c r="M1" s="3" t="s">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="N1" s="3" t="s">
-        <v>43</v>
+        <v>52</v>
       </c>
       <c r="O1" s="3" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
-        <v>55</v>
+        <v>64</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="C2" s="4">
         <v>1</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>45</v>
+        <v>54</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>46</v>
+        <v>55</v>
       </c>
       <c r="H2" s="4" t="s">
-        <v>47</v>
+        <v>56</v>
       </c>
       <c r="I2" s="4" t="s">
-        <v>48</v>
+        <v>57</v>
       </c>
       <c r="J2" s="4" t="s">
-        <v>49</v>
+        <v>58</v>
       </c>
       <c r="K2" s="4" t="s">
-        <v>50</v>
+        <v>59</v>
       </c>
       <c r="L2" s="4" t="s">
-        <v>51</v>
+        <v>60</v>
       </c>
       <c r="M2" s="4" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="N2" s="4" t="s">
-        <v>53</v>
+        <v>62</v>
       </c>
       <c r="O2" s="4" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
     </row>
   </sheetData>
@@ -1384,60 +1518,60 @@
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>58</v>
+        <v>67</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>37</v>
+        <v>46</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>38</v>
+        <v>47</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>59</v>
+        <v>68</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>60</v>
+        <v>69</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>61</v>
+        <v>70</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="J1" s="3" t="s">
-        <v>16</v>
+        <v>3</v>
       </c>
       <c r="K1" s="3" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
-        <v>62</v>
+        <v>71</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>63</v>
+        <v>72</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>64</v>
+        <v>73</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>65</v>
+        <v>74</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>66</v>
+        <v>75</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>67</v>
+        <v>76</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>68</v>
+        <v>77</v>
       </c>
       <c r="H2" s="4" t="s">
-        <v>69</v>
+        <v>78</v>
       </c>
       <c r="I2" s="4">
         <v>1.28</v>
@@ -1446,7 +1580,7 @@
         <v>22224</v>
       </c>
       <c r="K2" s="4" t="s">
-        <v>70</v>
+        <v>79</v>
       </c>
     </row>
   </sheetData>
@@ -1473,57 +1607,57 @@
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>71</v>
+        <v>80</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>72</v>
+        <v>81</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>58</v>
+        <v>67</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>37</v>
+        <v>46</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>38</v>
+        <v>47</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>59</v>
+        <v>68</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>60</v>
+        <v>69</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
-        <v>73</v>
+        <v>82</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>74</v>
+        <v>83</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>75</v>
+        <v>84</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>76</v>
+        <v>85</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>47</v>
+        <v>56</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>48</v>
+        <v>57</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>49</v>
+        <v>58</v>
       </c>
       <c r="H2" s="4" t="s">
-        <v>77</v>
+        <v>86</v>
       </c>
       <c r="I2" s="4" t="s">
-        <v>78</v>
+        <v>87</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Uodated: Review comments - code refactor - Web & Mobile Scenarios.
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/EnterpriseTestData.xlsx
+++ b/src/test/resources/testdata/EnterpriseTestData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/7717805a7dbae679/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="11_A180A8D17879FCD29DF161CB5464D75B08B36FDF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A10309DB-2934-4B9A-9157-FF2D155A5BAA}"/>
+  <xr:revisionPtr revIDLastSave="10" documentId="11_A180A8D17879FCD29DF161CB5464D75B08B36FDF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{82983F0B-D03C-43F8-8B3E-3DECD5776940}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="7" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="7" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="LoginData" sheetId="1" r:id="rId1"/>
@@ -332,7 +332,7 @@
     <t>New user registration with unique runtime-suffixed username</t>
   </si>
   <si>
-    <t>qa_morganalex_99_</t>
+    <t>ameam</t>
   </si>
 </sst>
 </file>
@@ -421,6 +421,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -900,7 +904,7 @@
     <col min="6" max="7" width="10" customWidth="1"/>
     <col min="8" max="8" width="14" customWidth="1"/>
     <col min="9" max="9" width="12" customWidth="1"/>
-    <col min="10" max="10" width="20.77734375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="21" customWidth="1"/>
     <col min="11" max="11" width="16" customWidth="1"/>
     <col min="12" max="12" width="50" customWidth="1"/>
   </cols>

</xml_diff>

<commit_message>
Update - Continued with Error scenarios - Mobile Scenarios.
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/EnterpriseTestData.xlsx
+++ b/src/test/resources/testdata/EnterpriseTestData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/7717805a7dbae679/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10" documentId="11_A180A8D17879FCD29DF161CB5464D75B08B36FDF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{82983F0B-D03C-43F8-8B3E-3DECD5776940}"/>
+  <xr:revisionPtr revIDLastSave="31" documentId="11_A180A8D17879FCD29DF161CB5464D75B08B36FDF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F303C371-1D8B-4614-B737-78DEF0B44DDF}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="7" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="2" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="LoginData" sheetId="1" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="227" uniqueCount="112">
   <si>
     <t>TestCaseID</t>
   </si>
@@ -333,6 +333,39 @@
   </si>
   <si>
     <t>ameam</t>
+  </si>
+  <si>
+    <t>Checkout_002</t>
+  </si>
+  <si>
+    <t>245 Sub St</t>
+  </si>
+  <si>
+    <t>BillFullName</t>
+  </si>
+  <si>
+    <t>BillAddress1</t>
+  </si>
+  <si>
+    <t>BillCity</t>
+  </si>
+  <si>
+    <t>BillState</t>
+  </si>
+  <si>
+    <t>BillZip</t>
+  </si>
+  <si>
+    <t>BillCountry</t>
+  </si>
+  <si>
+    <t>Minneapolis</t>
+  </si>
+  <si>
+    <t>Minnesota</t>
+  </si>
+  <si>
+    <t>Complete checkout with diff billing address</t>
   </si>
 </sst>
 </file>
@@ -396,7 +429,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
@@ -406,6 +439,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1278,7 +1314,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:S3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -1291,10 +1327,14 @@
     <col min="10" max="10" width="20" customWidth="1"/>
     <col min="11" max="11" width="16" customWidth="1"/>
     <col min="12" max="12" width="14" customWidth="1"/>
-    <col min="13" max="13" width="44" customWidth="1"/>
+    <col min="13" max="14" width="16" customWidth="1"/>
+    <col min="15" max="16" width="12" customWidth="1"/>
+    <col min="17" max="17" width="10" customWidth="1"/>
+    <col min="18" max="18" width="16" customWidth="1"/>
+    <col min="19" max="19" width="44" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -1332,10 +1372,28 @@
         <v>52</v>
       </c>
       <c r="M1" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="N1" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="O1" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="P1" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="Q1" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="R1" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="S1" s="3" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>53</v>
       </c>
@@ -1373,11 +1431,89 @@
         <v>62</v>
       </c>
       <c r="M2" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="N2" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="O2" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="P2" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="Q2" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="R2" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="S2" s="4" t="s">
         <v>63</v>
+      </c>
+    </row>
+    <row r="3" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A3" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C3" s="4">
+        <v>2</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="I3" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="J3" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="K3" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="L3" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="M3" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="N3" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="O3" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="P3" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="Q3" s="5">
+        <v>54612</v>
+      </c>
+      <c r="R3" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="S3" s="4" t="s">
+        <v>111</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Update - Added Model pages to get data from excel.
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/EnterpriseTestData.xlsx
+++ b/src/test/resources/testdata/EnterpriseTestData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/7717805a7dbae679/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="31" documentId="11_A180A8D17879FCD29DF161CB5464D75B08B36FDF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F303C371-1D8B-4614-B737-78DEF0B44DDF}"/>
+  <xr:revisionPtr revIDLastSave="55" documentId="11_A180A8D17879FCD29DF161CB5464D75B08B36FDF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2ED2912F-8FB9-40E8-A34D-AADF7A26E299}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="2" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="7" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="LoginData" sheetId="1" r:id="rId1"/>
@@ -18,8 +18,8 @@
     <sheet name="AccountOpen" sheetId="3" r:id="rId3"/>
     <sheet name="MobileLoginData" sheetId="4" r:id="rId4"/>
     <sheet name="MobileCartData" sheetId="5" r:id="rId5"/>
-    <sheet name="MobileCheckoutData" sheetId="6" r:id="rId6"/>
-    <sheet name="MobileCheckoutGuestData" sheetId="7" r:id="rId7"/>
+    <sheet name="MobileCheckoutGuestData" sheetId="7" r:id="rId6"/>
+    <sheet name="MobileCheckoutData" sheetId="6" r:id="rId7"/>
     <sheet name="BillPayData" sheetId="8" r:id="rId8"/>
     <sheet name="UpdateContactData" sheetId="9" r:id="rId9"/>
     <sheet name="RequestLoanData" sheetId="10" r:id="rId10"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="227" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="264" uniqueCount="111">
   <si>
     <t>TestCaseID</t>
   </si>
@@ -167,9 +167,6 @@
     <t>FullName</t>
   </si>
   <si>
-    <t>Address1</t>
-  </si>
-  <si>
     <t>City</t>
   </si>
   <si>
@@ -236,9 +233,6 @@
     <t>Address</t>
   </si>
   <si>
-    <t>ZipCode</t>
-  </si>
-  <si>
     <t>Phone</t>
   </si>
   <si>
@@ -344,9 +338,6 @@
     <t>BillFullName</t>
   </si>
   <si>
-    <t>BillAddress1</t>
-  </si>
-  <si>
     <t>BillCity</t>
   </si>
   <si>
@@ -366,13 +357,19 @@
   </si>
   <si>
     <t>Complete checkout with diff billing address</t>
+  </si>
+  <si>
+    <t>CheckoutGuest_002</t>
+  </si>
+  <si>
+    <t>BillAddress</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -392,6 +389,12 @@
       <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -930,95 +933,103 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:M2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="3" width="12" customWidth="1"/>
     <col min="4" max="4" width="18" customWidth="1"/>
     <col min="5" max="5" width="12" customWidth="1"/>
-    <col min="6" max="7" width="10" customWidth="1"/>
-    <col min="8" max="8" width="14" customWidth="1"/>
-    <col min="9" max="9" width="12" customWidth="1"/>
-    <col min="10" max="10" width="21" customWidth="1"/>
-    <col min="11" max="11" width="16" customWidth="1"/>
-    <col min="12" max="12" width="50" customWidth="1"/>
+    <col min="6" max="6" width="10" customWidth="1"/>
+    <col min="7" max="7" width="16" customWidth="1"/>
+    <col min="8" max="8" width="10" customWidth="1"/>
+    <col min="9" max="9" width="14" customWidth="1"/>
+    <col min="10" max="10" width="12" customWidth="1"/>
+    <col min="11" max="11" width="21" customWidth="1"/>
+    <col min="12" max="12" width="16" customWidth="1"/>
+    <col min="13" max="13" width="50" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="D1" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I1" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="E1" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="I1" s="3" t="s">
+      <c r="J1" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="K1" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="L1" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="M1" s="3" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A2" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="B2" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="J1" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="K1" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="L1" s="3" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A2" s="4" t="s">
+      <c r="C2" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="D2" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="E2" s="4" t="s">
         <v>91</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="F2" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="G2" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="H2" s="4" t="s">
         <v>93</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="I2" s="4" t="s">
         <v>94</v>
       </c>
-      <c r="G2" s="4" t="s">
+      <c r="J2" s="4" t="s">
         <v>95</v>
-      </c>
-      <c r="H2" s="4" t="s">
-        <v>96</v>
-      </c>
-      <c r="I2" s="4" t="s">
-        <v>97</v>
-      </c>
-      <c r="J2" s="4" t="s">
-        <v>100</v>
       </c>
       <c r="K2" s="4" t="s">
         <v>98</v>
       </c>
       <c r="L2" s="4" t="s">
-        <v>99</v>
+        <v>96</v>
+      </c>
+      <c r="M2" s="4" t="s">
+        <v>97</v>
       </c>
     </row>
   </sheetData>
@@ -1313,6 +1324,230 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
+  <dimension ref="A1:U3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="20" customWidth="1"/>
+    <col min="2" max="2" width="22" customWidth="1"/>
+    <col min="3" max="3" width="10" customWidth="1"/>
+    <col min="4" max="5" width="14" customWidth="1"/>
+    <col min="6" max="7" width="16" customWidth="1"/>
+    <col min="8" max="9" width="12" customWidth="1"/>
+    <col min="10" max="10" width="10" customWidth="1"/>
+    <col min="11" max="11" width="16" customWidth="1"/>
+    <col min="12" max="12" width="20" customWidth="1"/>
+    <col min="13" max="13" width="16" customWidth="1"/>
+    <col min="14" max="14" width="14" customWidth="1"/>
+    <col min="15" max="16" width="16" customWidth="1"/>
+    <col min="17" max="18" width="12" customWidth="1"/>
+    <col min="19" max="19" width="10" customWidth="1"/>
+    <col min="20" max="20" width="16" customWidth="1"/>
+    <col min="21" max="21" width="59.6640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="K1" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="L1" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="M1" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="N1" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="O1" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="P1" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="Q1" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="R1" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="S1" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="T1" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="U1" s="3" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A2" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C2" s="4">
+        <v>1</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="H2" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="I2" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="J2" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="K2" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="L2" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="M2" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="N2" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="O2" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="P2" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="Q2" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="R2" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="S2" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="T2" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="U2" s="4" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="3" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A3" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C3" s="4">
+        <v>2</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="I3" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="J3" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="K3" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="L3" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="M3" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="N3" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="O3" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="P3" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="Q3" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="R3" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="S3" s="5">
+        <v>54612</v>
+      </c>
+      <c r="T3" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="U3" s="4" t="s">
+        <v>108</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:S3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1348,46 +1583,46 @@
         <v>44</v>
       </c>
       <c r="E1" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="F1" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="G1" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="H1" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="I1" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="J1" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="K1" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="K1" s="3" t="s">
+      <c r="L1" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="L1" s="3" t="s">
-        <v>52</v>
-      </c>
       <c r="M1" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="N1" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="O1" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="P1" s="3" t="s">
         <v>103</v>
       </c>
-      <c r="N1" s="3" t="s">
+      <c r="Q1" s="3" t="s">
         <v>104</v>
       </c>
-      <c r="O1" s="3" t="s">
+      <c r="R1" s="3" t="s">
         <v>105</v>
-      </c>
-      <c r="P1" s="3" t="s">
-        <v>106</v>
-      </c>
-      <c r="Q1" s="3" t="s">
-        <v>107</v>
-      </c>
-      <c r="R1" s="3" t="s">
-        <v>108</v>
       </c>
       <c r="S1" s="3" t="s">
         <v>5</v>
@@ -1395,7 +1630,7 @@
     </row>
     <row r="2" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B2" s="4" t="s">
         <v>39</v>
@@ -1404,57 +1639,57 @@
         <v>1</v>
       </c>
       <c r="D2" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="E2" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="F2" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="G2" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="G2" s="4" t="s">
+      <c r="H2" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="H2" s="4" t="s">
+      <c r="I2" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="I2" s="4" t="s">
+      <c r="J2" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="J2" s="4" t="s">
+      <c r="K2" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="K2" s="4" t="s">
+      <c r="L2" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="L2" s="4" t="s">
+      <c r="M2" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="N2" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="O2" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="P2" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="Q2" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="R2" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="S2" s="4" t="s">
         <v>62</v>
-      </c>
-      <c r="M2" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="N2" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="O2" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="P2" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="Q2" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="R2" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="S2" s="4" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="3" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="B3" s="4" t="s">
         <v>39</v>
@@ -1463,52 +1698,52 @@
         <v>2</v>
       </c>
       <c r="D3" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="E3" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="F3" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="F3" s="4" t="s">
+      <c r="G3" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="G3" s="4" t="s">
+      <c r="H3" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="H3" s="4" t="s">
+      <c r="I3" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="I3" s="4" t="s">
+      <c r="J3" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="J3" s="4" t="s">
+      <c r="K3" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="K3" s="4" t="s">
+      <c r="L3" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="L3" s="4" t="s">
-        <v>62</v>
-      </c>
       <c r="M3" s="4" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="N3" s="4" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="O3" s="4" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="P3" s="4" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="Q3" s="5">
         <v>54612</v>
       </c>
       <c r="R3" s="4" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="S3" s="4" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
     </row>
   </sheetData>
@@ -1517,127 +1752,9 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
-  <dimension ref="A1:O2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="20" customWidth="1"/>
-    <col min="2" max="2" width="22" customWidth="1"/>
-    <col min="3" max="3" width="10" customWidth="1"/>
-    <col min="4" max="5" width="14" customWidth="1"/>
-    <col min="6" max="7" width="16" customWidth="1"/>
-    <col min="8" max="9" width="12" customWidth="1"/>
-    <col min="10" max="10" width="10" customWidth="1"/>
-    <col min="11" max="11" width="16" customWidth="1"/>
-    <col min="12" max="12" width="20" customWidth="1"/>
-    <col min="13" max="13" width="16" customWidth="1"/>
-    <col min="14" max="14" width="14" customWidth="1"/>
-    <col min="15" max="15" width="48" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A1" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="I1" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="J1" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="K1" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="L1" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="M1" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="N1" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="O1" s="3" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A2" s="4" t="s">
-        <v>64</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="C2" s="4">
-        <v>1</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="F2" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="G2" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="H2" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="I2" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="J2" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="K2" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="L2" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="M2" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="N2" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="O2" s="4" t="s">
-        <v>65</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:L2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12.44140625" bestFit="1" customWidth="1"/>
@@ -1646,81 +1763,88 @@
     <col min="4" max="4" width="14.33203125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="9.44140625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="9.109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="16.88671875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="8.6640625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="14" customWidth="1"/>
-    <col min="11" max="11" width="26" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16" customWidth="1"/>
+    <col min="8" max="8" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="16.88671875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="8.6640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="14" customWidth="1"/>
+    <col min="12" max="12" width="26" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="C1" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="D1" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="H1" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="D1" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="F1" s="3" t="s">
+      <c r="I1" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="J1" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="L1" s="3" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A2" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="B2" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="I1" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="K1" s="3" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A2" s="4" t="s">
+      <c r="C2" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="D2" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="E2" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="F2" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="G2" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="H2" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="I2" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="G2" s="4" t="s">
+      <c r="J2" s="4">
+        <v>1.28</v>
+      </c>
+      <c r="K2" s="4">
+        <v>22224</v>
+      </c>
+      <c r="L2" s="4" t="s">
         <v>77</v>
-      </c>
-      <c r="H2" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="I2" s="4">
-        <v>1.28</v>
-      </c>
-      <c r="J2" s="4">
-        <v>22224</v>
-      </c>
-      <c r="K2" s="4" t="s">
-        <v>79</v>
       </c>
     </row>
   </sheetData>
@@ -1730,7 +1854,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:J2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -1738,66 +1862,73 @@
     <col min="4" max="4" width="16" customWidth="1"/>
     <col min="5" max="6" width="12" customWidth="1"/>
     <col min="7" max="7" width="10" customWidth="1"/>
-    <col min="8" max="8" width="14" customWidth="1"/>
-    <col min="9" max="9" width="40" customWidth="1"/>
+    <col min="8" max="8" width="16" customWidth="1"/>
+    <col min="9" max="9" width="14" customWidth="1"/>
+    <col min="10" max="10" width="40" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A2" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="B2" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="D1" s="3" t="s">
-        <v>67</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="I1" s="3" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A2" s="4" t="s">
+      <c r="C2" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="D2" s="4" t="s">
         <v>83</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="E2" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="H2" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="I2" s="4" t="s">
         <v>84</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="J2" s="4" t="s">
         <v>85</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="F2" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="G2" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="H2" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="I2" s="4" t="s">
-        <v>87</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix: force flush git cache and apply gitignore
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/EnterpriseTestData.xlsx
+++ b/src/test/resources/testdata/EnterpriseTestData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/7717805a7dbae679/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="55" documentId="11_A180A8D17879FCD29DF161CB5464D75B08B36FDF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2ED2912F-8FB9-40E8-A34D-AADF7A26E299}"/>
+  <xr:revisionPtr revIDLastSave="60" documentId="11_A180A8D17879FCD29DF161CB5464D75B08B36FDF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D8E5F4E1-AD47-4546-AC28-D7CF95A15B23}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="7" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="6" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="LoginData" sheetId="1" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="264" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="264" uniqueCount="112">
   <si>
     <t>TestCaseID</t>
   </si>
@@ -209,9 +209,6 @@
     <t>United States</t>
   </si>
   <si>
-    <t>4111111111111111</t>
-  </si>
-  <si>
     <t>12/28</t>
   </si>
   <si>
@@ -363,6 +360,12 @@
   </si>
   <si>
     <t>BillAddress</t>
+  </si>
+  <si>
+    <t>4111 1111 1111 1111</t>
+  </si>
+  <si>
+    <t>4111 1111 1111 2222</t>
   </si>
 </sst>
 </file>
@@ -460,10 +463,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -955,13 +954,13 @@
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="C1" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="C1" s="3" t="s">
-        <v>79</v>
-      </c>
       <c r="D1" s="3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E1" s="3" t="s">
         <v>45</v>
@@ -976,10 +975,10 @@
         <v>47</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="J1" s="3" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="K1" s="3" t="s">
         <v>12</v>
@@ -993,43 +992,43 @@
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="B2" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="C2" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="D2" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="E2" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="F2" s="4" t="s">
         <v>91</v>
-      </c>
-      <c r="F2" s="4" t="s">
-        <v>92</v>
       </c>
       <c r="G2" s="4" t="s">
         <v>58</v>
       </c>
       <c r="H2" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="I2" s="4" t="s">
         <v>93</v>
       </c>
-      <c r="I2" s="4" t="s">
+      <c r="J2" s="4" t="s">
         <v>94</v>
       </c>
-      <c r="J2" s="4" t="s">
+      <c r="K2" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="L2" s="4" t="s">
         <v>95</v>
       </c>
-      <c r="K2" s="4" t="s">
-        <v>98</v>
-      </c>
-      <c r="L2" s="4" t="s">
+      <c r="M2" s="4" t="s">
         <v>96</v>
-      </c>
-      <c r="M2" s="4" t="s">
-        <v>97</v>
       </c>
     </row>
   </sheetData>
@@ -1336,7 +1335,7 @@
     <col min="8" max="9" width="12" customWidth="1"/>
     <col min="10" max="10" width="10" customWidth="1"/>
     <col min="11" max="11" width="16" customWidth="1"/>
-    <col min="12" max="12" width="20" customWidth="1"/>
+    <col min="12" max="12" width="22" customWidth="1"/>
     <col min="13" max="13" width="16" customWidth="1"/>
     <col min="14" max="14" width="14" customWidth="1"/>
     <col min="15" max="16" width="16" customWidth="1"/>
@@ -1366,7 +1365,7 @@
         <v>44</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="H1" s="3" t="s">
         <v>45</v>
@@ -1390,22 +1389,22 @@
         <v>51</v>
       </c>
       <c r="O1" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="P1" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="Q1" s="3" t="s">
         <v>101</v>
       </c>
-      <c r="P1" s="3" t="s">
-        <v>110</v>
-      </c>
-      <c r="Q1" s="3" t="s">
+      <c r="R1" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="R1" s="3" t="s">
+      <c r="S1" s="3" t="s">
         <v>103</v>
       </c>
-      <c r="S1" s="3" t="s">
+      <c r="T1" s="3" t="s">
         <v>104</v>
-      </c>
-      <c r="T1" s="3" t="s">
-        <v>105</v>
       </c>
       <c r="U1" s="3" t="s">
         <v>5</v>
@@ -1413,7 +1412,7 @@
     </row>
     <row r="2" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B2" s="4" t="s">
         <v>39</v>
@@ -1446,13 +1445,13 @@
         <v>58</v>
       </c>
       <c r="L2" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="M2" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="M2" s="4" t="s">
+      <c r="N2" s="4" t="s">
         <v>60</v>
-      </c>
-      <c r="N2" s="4" t="s">
-        <v>61</v>
       </c>
       <c r="O2" s="4" t="s">
         <v>53</v>
@@ -1473,12 +1472,12 @@
         <v>58</v>
       </c>
       <c r="U2" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="3" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B3" s="4" t="s">
         <v>39</v>
@@ -1511,25 +1510,25 @@
         <v>58</v>
       </c>
       <c r="L3" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="M3" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="M3" s="4" t="s">
+      <c r="N3" s="4" t="s">
         <v>60</v>
-      </c>
-      <c r="N3" s="4" t="s">
-        <v>61</v>
       </c>
       <c r="O3" s="4" t="s">
         <v>53</v>
       </c>
       <c r="P3" s="4" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="Q3" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="R3" s="4" t="s">
         <v>106</v>
-      </c>
-      <c r="R3" s="4" t="s">
-        <v>107</v>
       </c>
       <c r="S3" s="5">
         <v>54612</v>
@@ -1538,7 +1537,7 @@
         <v>58</v>
       </c>
       <c r="U3" s="4" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
   </sheetData>
@@ -1583,7 +1582,7 @@
         <v>44</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="F1" s="3" t="s">
         <v>45</v>
@@ -1607,22 +1606,22 @@
         <v>51</v>
       </c>
       <c r="M1" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="N1" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="O1" s="3" t="s">
         <v>101</v>
       </c>
-      <c r="N1" s="3" t="s">
-        <v>110</v>
-      </c>
-      <c r="O1" s="3" t="s">
+      <c r="P1" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="P1" s="3" t="s">
+      <c r="Q1" s="3" t="s">
         <v>103</v>
       </c>
-      <c r="Q1" s="3" t="s">
+      <c r="R1" s="3" t="s">
         <v>104</v>
-      </c>
-      <c r="R1" s="3" t="s">
-        <v>105</v>
       </c>
       <c r="S1" s="3" t="s">
         <v>5</v>
@@ -1657,13 +1656,13 @@
         <v>58</v>
       </c>
       <c r="J2" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="K2" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="K2" s="4" t="s">
+      <c r="L2" s="4" t="s">
         <v>60</v>
-      </c>
-      <c r="L2" s="4" t="s">
-        <v>61</v>
       </c>
       <c r="M2" s="4" t="s">
         <v>53</v>
@@ -1684,12 +1683,12 @@
         <v>58</v>
       </c>
       <c r="S2" s="4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="3" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B3" s="4" t="s">
         <v>39</v>
@@ -1716,25 +1715,25 @@
         <v>58</v>
       </c>
       <c r="J3" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="K3" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="K3" s="4" t="s">
+      <c r="L3" s="4" t="s">
         <v>60</v>
-      </c>
-      <c r="L3" s="4" t="s">
-        <v>61</v>
       </c>
       <c r="M3" s="4" t="s">
         <v>53</v>
       </c>
       <c r="N3" s="4" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="O3" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="P3" s="4" t="s">
         <v>106</v>
-      </c>
-      <c r="P3" s="4" t="s">
-        <v>107</v>
       </c>
       <c r="Q3" s="5">
         <v>54612</v>
@@ -1743,7 +1742,7 @@
         <v>58</v>
       </c>
       <c r="S3" s="4" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
   </sheetData>
@@ -1776,10 +1775,10 @@
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="C1" s="3" t="s">
         <v>65</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>66</v>
       </c>
       <c r="D1" s="3" t="s">
         <v>45</v>
@@ -1794,10 +1793,10 @@
         <v>48</v>
       </c>
       <c r="H1" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="I1" s="3" t="s">
         <v>67</v>
-      </c>
-      <c r="I1" s="3" t="s">
-        <v>68</v>
       </c>
       <c r="J1" s="3" t="s">
         <v>27</v>
@@ -1811,31 +1810,31 @@
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="B2" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="C2" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="D2" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="E2" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="F2" s="4" t="s">
         <v>73</v>
-      </c>
-      <c r="F2" s="4" t="s">
-        <v>74</v>
       </c>
       <c r="G2" s="4" t="s">
         <v>58</v>
       </c>
       <c r="H2" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="I2" s="4" t="s">
         <v>75</v>
-      </c>
-      <c r="I2" s="4" t="s">
-        <v>76</v>
       </c>
       <c r="J2" s="4">
         <v>1.28</v>
@@ -1844,7 +1843,7 @@
         <v>22224</v>
       </c>
       <c r="L2" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
   </sheetData>
@@ -1872,13 +1871,13 @@
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="C1" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="C1" s="3" t="s">
-        <v>79</v>
-      </c>
       <c r="D1" s="3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E1" s="3" t="s">
         <v>45</v>
@@ -1893,7 +1892,7 @@
         <v>48</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="J1" s="3" t="s">
         <v>5</v>
@@ -1901,16 +1900,16 @@
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="B2" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="C2" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="D2" s="4" t="s">
         <v>82</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>83</v>
       </c>
       <c r="E2" s="4" t="s">
         <v>55</v>
@@ -1925,10 +1924,10 @@
         <v>58</v>
       </c>
       <c r="I2" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="J2" s="4" t="s">
         <v>84</v>
-      </c>
-      <c r="J2" s="4" t="s">
-        <v>85</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Enhance Sort feature results verify in mobile app.
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/EnterpriseTestData.xlsx
+++ b/src/test/resources/testdata/EnterpriseTestData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/7717805a7dbae679/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="60" documentId="11_A180A8D17879FCD29DF161CB5464D75B08B36FDF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D8E5F4E1-AD47-4546-AC28-D7CF95A15B23}"/>
+  <xr:revisionPtr revIDLastSave="68" documentId="11_A180A8D17879FCD29DF161CB5464D75B08B36FDF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7497C1FE-347C-4105-A41C-45C2205064F1}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="6" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="5" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="LoginData" sheetId="1" r:id="rId1"/>
@@ -158,12 +158,6 @@
     <t>Cart_002</t>
   </si>
   <si>
-    <t>Sauce Labs Bike Light</t>
-  </si>
-  <si>
-    <t>Add product intended for removal scenario</t>
-  </si>
-  <si>
     <t>FullName</t>
   </si>
   <si>
@@ -366,6 +360,12 @@
   </si>
   <si>
     <t>4111 1111 1111 2222</t>
+  </si>
+  <si>
+    <t>Sauce Labs Backpack (yellow)</t>
+  </si>
+  <si>
+    <t>Add single product with quantity to cart — color-variant SKU further down the catalog, requires scroll</t>
   </si>
 </sst>
 </file>
@@ -463,6 +463,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -954,31 +958,31 @@
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="E1" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="H1" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="F1" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>47</v>
-      </c>
       <c r="I1" s="3" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="J1" s="3" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="K1" s="3" t="s">
         <v>12</v>
@@ -992,43 +996,43 @@
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="C2" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="D2" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="E2" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="F2" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="G2" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="H2" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="I2" s="4" t="s">
         <v>91</v>
       </c>
-      <c r="G2" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="H2" s="4" t="s">
+      <c r="J2" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="I2" s="4" t="s">
+      <c r="K2" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="L2" s="4" t="s">
         <v>93</v>
       </c>
-      <c r="J2" s="4" t="s">
+      <c r="M2" s="4" t="s">
         <v>94</v>
-      </c>
-      <c r="K2" s="4" t="s">
-        <v>97</v>
-      </c>
-      <c r="L2" s="4" t="s">
-        <v>95</v>
-      </c>
-      <c r="M2" s="4" t="s">
-        <v>96</v>
       </c>
     </row>
   </sheetData>
@@ -1270,9 +1274,9 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17" customWidth="1"/>
-    <col min="2" max="2" width="24" customWidth="1"/>
+    <col min="2" max="2" width="28.6640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12" customWidth="1"/>
-    <col min="4" max="4" width="42" customWidth="1"/>
+    <col min="4" max="4" width="91.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
@@ -1308,13 +1312,13 @@
         <v>41</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>42</v>
+        <v>110</v>
       </c>
       <c r="C3" s="4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>43</v>
+        <v>111</v>
       </c>
     </row>
   </sheetData>
@@ -1328,7 +1332,7 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
-    <col min="2" max="2" width="22" customWidth="1"/>
+    <col min="2" max="2" width="28.6640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10" customWidth="1"/>
     <col min="4" max="5" width="14" customWidth="1"/>
     <col min="6" max="7" width="16" customWidth="1"/>
@@ -1362,49 +1366,49 @@
         <v>13</v>
       </c>
       <c r="F1" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="I1" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="G1" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="H1" s="3" t="s">
+      <c r="J1" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="K1" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="L1" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="K1" s="3" t="s">
+      <c r="M1" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="L1" s="3" t="s">
+      <c r="N1" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="M1" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="N1" s="3" t="s">
-        <v>51</v>
-      </c>
       <c r="O1" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="P1" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="Q1" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="R1" s="3" t="s">
         <v>100</v>
       </c>
-      <c r="P1" s="3" t="s">
-        <v>109</v>
-      </c>
-      <c r="Q1" s="3" t="s">
+      <c r="S1" s="3" t="s">
         <v>101</v>
       </c>
-      <c r="R1" s="3" t="s">
+      <c r="T1" s="3" t="s">
         <v>102</v>
-      </c>
-      <c r="S1" s="3" t="s">
-        <v>103</v>
-      </c>
-      <c r="T1" s="3" t="s">
-        <v>104</v>
       </c>
       <c r="U1" s="3" t="s">
         <v>5</v>
@@ -1412,7 +1416,7 @@
     </row>
     <row r="2" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="B2" s="4" t="s">
         <v>39</v>
@@ -1427,60 +1431,60 @@
         <v>16</v>
       </c>
       <c r="F2" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="H2" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="G2" s="4" t="s">
+      <c r="I2" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="H2" s="4" t="s">
+      <c r="J2" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="I2" s="4" t="s">
+      <c r="K2" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="J2" s="4" t="s">
+      <c r="L2" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="M2" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="K2" s="4" t="s">
+      <c r="N2" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="L2" s="4" t="s">
-        <v>110</v>
-      </c>
-      <c r="M2" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="N2" s="4" t="s">
-        <v>60</v>
-      </c>
       <c r="O2" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="P2" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="Q2" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="P2" s="4" t="s">
+      <c r="R2" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="Q2" s="4" t="s">
+      <c r="S2" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="R2" s="4" t="s">
+      <c r="T2" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="S2" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="T2" s="4" t="s">
-        <v>58</v>
-      </c>
       <c r="U2" s="4" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
     <row r="3" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>39</v>
+        <v>110</v>
       </c>
       <c r="C3" s="4">
         <v>2</v>
@@ -1492,52 +1496,52 @@
         <v>16</v>
       </c>
       <c r="F3" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="H3" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="G3" s="4" t="s">
+      <c r="I3" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="H3" s="4" t="s">
+      <c r="J3" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="I3" s="4" t="s">
+      <c r="K3" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="J3" s="4" t="s">
+      <c r="L3" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="M3" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="K3" s="4" t="s">
+      <c r="N3" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="L3" s="4" t="s">
-        <v>111</v>
-      </c>
-      <c r="M3" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="N3" s="4" t="s">
-        <v>60</v>
-      </c>
       <c r="O3" s="4" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="P3" s="4" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="Q3" s="4" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="R3" s="4" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="S3" s="5">
         <v>54612</v>
       </c>
       <c r="T3" s="4" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="U3" s="4" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
     </row>
   </sheetData>
@@ -1552,7 +1556,7 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
-    <col min="2" max="2" width="22" customWidth="1"/>
+    <col min="2" max="2" width="28.6640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10" customWidth="1"/>
     <col min="4" max="5" width="16" customWidth="1"/>
     <col min="6" max="7" width="12" customWidth="1"/>
@@ -1579,49 +1583,49 @@
         <v>37</v>
       </c>
       <c r="D1" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="G1" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="E1" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="F1" s="3" t="s">
+      <c r="H1" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="I1" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="J1" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="K1" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="L1" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="K1" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="L1" s="3" t="s">
-        <v>51</v>
-      </c>
       <c r="M1" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="N1" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="O1" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="P1" s="3" t="s">
         <v>100</v>
       </c>
-      <c r="N1" s="3" t="s">
-        <v>109</v>
-      </c>
-      <c r="O1" s="3" t="s">
+      <c r="Q1" s="3" t="s">
         <v>101</v>
       </c>
-      <c r="P1" s="3" t="s">
+      <c r="R1" s="3" t="s">
         <v>102</v>
-      </c>
-      <c r="Q1" s="3" t="s">
-        <v>103</v>
-      </c>
-      <c r="R1" s="3" t="s">
-        <v>104</v>
       </c>
       <c r="S1" s="3" t="s">
         <v>5</v>
@@ -1629,7 +1633,7 @@
     </row>
     <row r="2" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B2" s="4" t="s">
         <v>39</v>
@@ -1638,111 +1642,111 @@
         <v>1</v>
       </c>
       <c r="D2" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="F2" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="G2" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="H2" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="G2" s="4" t="s">
+      <c r="I2" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="H2" s="4" t="s">
+      <c r="J2" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="K2" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="I2" s="4" t="s">
+      <c r="L2" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="J2" s="4" t="s">
-        <v>110</v>
-      </c>
-      <c r="K2" s="4" t="s">
+      <c r="M2" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="N2" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="O2" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="P2" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="Q2" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="R2" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="S2" s="4" t="s">
         <v>59</v>
-      </c>
-      <c r="L2" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="M2" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="N2" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="O2" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="P2" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="Q2" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="R2" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="S2" s="4" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="3" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>39</v>
+        <v>110</v>
       </c>
       <c r="C3" s="4">
         <v>2</v>
       </c>
       <c r="D3" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="F3" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="G3" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="F3" s="4" t="s">
+      <c r="H3" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="G3" s="4" t="s">
+      <c r="I3" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="H3" s="4" t="s">
+      <c r="J3" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="K3" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="I3" s="4" t="s">
+      <c r="L3" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="J3" s="4" t="s">
-        <v>111</v>
-      </c>
-      <c r="K3" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="L3" s="4" t="s">
-        <v>60</v>
-      </c>
       <c r="M3" s="4" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="N3" s="4" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="O3" s="4" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="P3" s="4" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="Q3" s="5">
         <v>54612</v>
       </c>
       <c r="R3" s="4" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="S3" s="4" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
     </row>
   </sheetData>
@@ -1775,28 +1779,28 @@
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="H1" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="I1" s="3" t="s">
         <v>65</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="I1" s="3" t="s">
-        <v>67</v>
       </c>
       <c r="J1" s="3" t="s">
         <v>27</v>
@@ -1810,31 +1814,31 @@
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="C2" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="D2" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="E2" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="F2" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="G2" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="H2" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="I2" s="4" t="s">
         <v>73</v>
-      </c>
-      <c r="G2" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="H2" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="I2" s="4" t="s">
-        <v>75</v>
       </c>
       <c r="J2" s="4">
         <v>1.28</v>
@@ -1843,7 +1847,7 @@
         <v>22224</v>
       </c>
       <c r="L2" s="4" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
     </row>
   </sheetData>
@@ -1871,28 +1875,28 @@
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="E1" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="G1" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="H1" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="G1" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>48</v>
-      </c>
       <c r="I1" s="3" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="J1" s="3" t="s">
         <v>5</v>
@@ -1900,34 +1904,34 @@
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="C2" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="D2" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="E2" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="H2" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="I2" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="J2" s="4" t="s">
         <v>82</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="F2" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="G2" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="H2" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="I2" s="4" t="s">
-        <v>83</v>
-      </c>
-      <c r="J2" s="4" t="s">
-        <v>84</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added few scenarios to Web app.
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/EnterpriseTestData.xlsx
+++ b/src/test/resources/testdata/EnterpriseTestData.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/7717805a7dbae679/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Automation\playwright-cucumber-testng-framework\src\test\resources\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="68" documentId="11_A180A8D17879FCD29DF161CB5464D75B08B36FDF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7497C1FE-347C-4105-A41C-45C2205064F1}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99547068-1265-4286-944C-01A7634666EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="5" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="5" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="LoginData" sheetId="1" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="264" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="268" uniqueCount="110">
   <si>
     <t>TestCaseID</t>
   </si>
@@ -89,24 +89,12 @@
     <t>Login_002</t>
   </si>
   <si>
-    <t>martha</t>
-  </si>
-  <si>
-    <t>demo123</t>
-  </si>
-  <si>
     <t>Valid account iteration 2</t>
   </si>
   <si>
     <t>Login_003</t>
   </si>
   <si>
-    <t>robert</t>
-  </si>
-  <si>
-    <t>testing</t>
-  </si>
-  <si>
     <t>Valid account iteration 3</t>
   </si>
   <si>
@@ -366,6 +354,12 @@
   </si>
   <si>
     <t>Add single product with quantity to cart — color-variant SKU further down the catalog, requires scroll</t>
+  </si>
+  <si>
+    <t>AcctOpen_003</t>
+  </si>
+  <si>
+    <t>Insufficient funds negative test, unconfirmed against live app</t>
   </si>
 </sst>
 </file>
@@ -463,10 +457,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -827,27 +817,27 @@
         <v>18</v>
       </c>
       <c r="B3" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D3" s="2" t="s">
         <v>19</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
     </row>
   </sheetData>
@@ -958,31 +948,31 @@
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="J1" s="3" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="K1" s="3" t="s">
         <v>12</v>
@@ -996,43 +986,43 @@
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="E2" s="4" t="s">
         <v>84</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="F2" s="4" t="s">
         <v>85</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="G2" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="H2" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="I2" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="J2" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="K2" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="L2" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="G2" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="H2" s="4" t="s">
+      <c r="M2" s="4" t="s">
         <v>90</v>
-      </c>
-      <c r="I2" s="4" t="s">
-        <v>91</v>
-      </c>
-      <c r="J2" s="4" t="s">
-        <v>92</v>
-      </c>
-      <c r="K2" s="4" t="s">
-        <v>95</v>
-      </c>
-      <c r="L2" s="4" t="s">
-        <v>93</v>
-      </c>
-      <c r="M2" s="4" t="s">
-        <v>94</v>
       </c>
     </row>
   </sheetData>
@@ -1068,10 +1058,10 @@
         <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>5</v>
@@ -1079,7 +1069,7 @@
     </row>
     <row r="2" spans="1:7" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>15</v>
@@ -1097,18 +1087,18 @@
         <v>10</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="D3" s="2">
         <v>56634</v>
@@ -1120,7 +1110,7 @@
         <v>25.5</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
     </row>
   </sheetData>
@@ -1130,14 +1120,14 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17.77734375" customWidth="1"/>
     <col min="2" max="2" width="12.21875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="21" customWidth="1"/>
     <col min="4" max="4" width="21.5546875" customWidth="1"/>
-    <col min="5" max="5" width="30.109375" customWidth="1"/>
+    <col min="5" max="5" width="75.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -1159,7 +1149,7 @@
     </row>
     <row r="2" spans="1:5" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>15</v>
@@ -1171,24 +1161,41 @@
         <v>22224</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="D3" s="2">
         <v>56634</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>35</v>
+        <v>31</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D4" s="2">
+        <v>12345</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>109</v>
       </c>
     </row>
   </sheetData>
@@ -1239,27 +1246,27 @@
         <v>18</v>
       </c>
       <c r="B3" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D3" s="2" t="s">
         <v>19</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
     </row>
   </sheetData>
@@ -1284,10 +1291,10 @@
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="D1" s="3" t="s">
         <v>5</v>
@@ -1295,30 +1302,30 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="C2" s="4">
         <v>2</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="C3" s="4">
         <v>2</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
     </row>
   </sheetData>
@@ -1354,10 +1361,10 @@
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="D1" s="3" t="s">
         <v>12</v>
@@ -1366,49 +1373,49 @@
         <v>13</v>
       </c>
       <c r="F1" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="K1" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="G1" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="H1" s="3" t="s">
+      <c r="L1" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="M1" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="N1" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="K1" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="L1" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="M1" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="N1" s="3" t="s">
-        <v>49</v>
-      </c>
       <c r="O1" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="P1" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="Q1" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="R1" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="S1" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="T1" s="3" t="s">
         <v>98</v>
-      </c>
-      <c r="P1" s="3" t="s">
-        <v>107</v>
-      </c>
-      <c r="Q1" s="3" t="s">
-        <v>99</v>
-      </c>
-      <c r="R1" s="3" t="s">
-        <v>100</v>
-      </c>
-      <c r="S1" s="3" t="s">
-        <v>101</v>
-      </c>
-      <c r="T1" s="3" t="s">
-        <v>102</v>
       </c>
       <c r="U1" s="3" t="s">
         <v>5</v>
@@ -1416,10 +1423,10 @@
     </row>
     <row r="2" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="C2" s="4">
         <v>1</v>
@@ -1431,60 +1438,60 @@
         <v>16</v>
       </c>
       <c r="F2" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="H2" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="I2" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="J2" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="G2" s="4" t="s">
+      <c r="K2" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="H2" s="4" t="s">
+      <c r="L2" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="M2" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="I2" s="4" t="s">
+      <c r="N2" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="J2" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="K2" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="L2" s="4" t="s">
-        <v>108</v>
-      </c>
-      <c r="M2" s="4" t="s">
+      <c r="O2" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="P2" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="Q2" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="R2" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="S2" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="T2" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="U2" s="4" t="s">
         <v>57</v>
-      </c>
-      <c r="N2" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="O2" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="P2" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="Q2" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="R2" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="S2" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="T2" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="U2" s="4" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="3" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="B3" s="4" t="s">
         <v>106</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>110</v>
       </c>
       <c r="C3" s="4">
         <v>2</v>
@@ -1496,52 +1503,52 @@
         <v>16</v>
       </c>
       <c r="F3" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="I3" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="J3" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="G3" s="4" t="s">
+      <c r="K3" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="H3" s="4" t="s">
+      <c r="L3" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="M3" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="I3" s="4" t="s">
+      <c r="N3" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="J3" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="K3" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="L3" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="M3" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="N3" s="4" t="s">
-        <v>58</v>
-      </c>
       <c r="O3" s="4" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="P3" s="4" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="Q3" s="4" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="R3" s="4" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="S3" s="5">
         <v>54612</v>
       </c>
       <c r="T3" s="4" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="U3" s="4" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
     </row>
   </sheetData>
@@ -1577,55 +1584,55 @@
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="D1" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="I1" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="E1" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="F1" s="3" t="s">
+      <c r="J1" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="K1" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="L1" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="I1" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="J1" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="K1" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="L1" s="3" t="s">
-        <v>49</v>
-      </c>
       <c r="M1" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="N1" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="O1" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="P1" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="Q1" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="R1" s="3" t="s">
         <v>98</v>
-      </c>
-      <c r="N1" s="3" t="s">
-        <v>107</v>
-      </c>
-      <c r="O1" s="3" t="s">
-        <v>99</v>
-      </c>
-      <c r="P1" s="3" t="s">
-        <v>100</v>
-      </c>
-      <c r="Q1" s="3" t="s">
-        <v>101</v>
-      </c>
-      <c r="R1" s="3" t="s">
-        <v>102</v>
       </c>
       <c r="S1" s="3" t="s">
         <v>5</v>
@@ -1633,120 +1640,120 @@
     </row>
     <row r="2" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="C2" s="4">
         <v>1</v>
       </c>
       <c r="D2" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="H2" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="I2" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="J2" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="K2" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="G2" s="4" t="s">
+      <c r="L2" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="H2" s="4" t="s">
+      <c r="M2" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="N2" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="O2" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="P2" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="Q2" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="R2" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="S2" s="4" t="s">
         <v>55</v>
-      </c>
-      <c r="I2" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="J2" s="4" t="s">
-        <v>108</v>
-      </c>
-      <c r="K2" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="L2" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="M2" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="N2" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="O2" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="P2" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="Q2" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="R2" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="S2" s="4" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="3" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="C3" s="4">
         <v>2</v>
       </c>
       <c r="D3" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="H3" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="I3" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="F3" s="4" t="s">
+      <c r="J3" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="K3" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="G3" s="4" t="s">
+      <c r="L3" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="H3" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="I3" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="J3" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="K3" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="L3" s="4" t="s">
-        <v>58</v>
-      </c>
       <c r="M3" s="4" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="N3" s="4" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="O3" s="4" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="P3" s="4" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="Q3" s="5">
         <v>54612</v>
       </c>
       <c r="R3" s="4" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="S3" s="4" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
     </row>
   </sheetData>
@@ -1779,31 +1786,31 @@
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="J1" s="3" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="K1" s="3" t="s">
         <v>3</v>
@@ -1814,31 +1821,31 @@
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="E2" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="F2" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="G2" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="H2" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="I2" s="4" t="s">
         <v>69</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="F2" s="4" t="s">
-        <v>71</v>
-      </c>
-      <c r="G2" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="H2" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="I2" s="4" t="s">
-        <v>73</v>
       </c>
       <c r="J2" s="4">
         <v>1.28</v>
@@ -1847,7 +1854,7 @@
         <v>22224</v>
       </c>
       <c r="L2" s="4" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
     </row>
   </sheetData>
@@ -1875,28 +1882,28 @@
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="J1" s="3" t="s">
         <v>5</v>
@@ -1904,34 +1911,34 @@
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="H2" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="I2" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="J2" s="4" t="s">
         <v>78</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>79</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>80</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="F2" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="G2" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="H2" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="I2" s="4" t="s">
-        <v>81</v>
-      </c>
-      <c r="J2" s="4" t="s">
-        <v>82</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add : Some more scenarios to Web App.
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/EnterpriseTestData.xlsx
+++ b/src/test/resources/testdata/EnterpriseTestData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Automation\playwright-cucumber-testng-framework\src\test\resources\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99547068-1265-4286-944C-01A7634666EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{725E1A3A-9A1F-4A6A-97C4-4A9B80CAFCE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="5" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="LoginData" sheetId="1" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="268" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="264" uniqueCount="108">
   <si>
     <t>TestCaseID</t>
   </si>
@@ -354,12 +354,6 @@
   </si>
   <si>
     <t>Add single product with quantity to cart — color-variant SKU further down the catalog, requires scroll</t>
-  </si>
-  <si>
-    <t>AcctOpen_003</t>
-  </si>
-  <si>
-    <t>Insufficient funds negative test, unconfirmed against live app</t>
   </si>
 </sst>
 </file>
@@ -1120,7 +1114,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17.77734375" customWidth="1"/>
@@ -1179,23 +1173,6 @@
       </c>
       <c r="E3" s="2" t="s">
         <v>31</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="D4" s="2">
-        <v>12345</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>109</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add : Minor changes to Web App.
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/EnterpriseTestData.xlsx
+++ b/src/test/resources/testdata/EnterpriseTestData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Automation\playwright-cucumber-testng-framework\src\test\resources\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{725E1A3A-9A1F-4A6A-97C4-4A9B80CAFCE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71BEDDB3-AA79-4BCE-9806-0129997AD7B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="2" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="LoginData" sheetId="1" r:id="rId1"/>
@@ -1623,7 +1623,7 @@
         <v>35</v>
       </c>
       <c r="C2" s="4">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D2" s="4" t="s">
         <v>47</v>
@@ -1682,7 +1682,7 @@
         <v>106</v>
       </c>
       <c r="C3" s="4">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D3" s="4" t="s">
         <v>47</v>

</xml_diff>